<commit_message>
Add Mega Millions live tracker and update Powerball data
- Add megamillions_lottery.py: fetches live draws from NY Open Data API,
  stores history in megamillions_game.xlsx, and suggests numbers using
  hot and hot+fresh frequency-based strategies (mirrors powerball_lottery.py)
- Add megamillions_game.xlsx: auto-generated data store with 100 historical draws
- Update powerball_game.xlsx with latest draw data

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/powerball_game.xlsx
+++ b/powerball_game.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,61 +413,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1949"/>
+  <dimension ref="A1:K1951"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>GameName</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Month</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Num1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Num2</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Num3</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Num4</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Num5</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>powerball</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Power Play</t>
         </is>
@@ -72139,6 +72127,80 @@
       </c>
       <c r="K1949" t="n">
         <v>3</v>
+      </c>
+    </row>
+    <row r="1950">
+      <c r="A1950" t="inlineStr">
+        <is>
+          <t>Powerball</t>
+        </is>
+      </c>
+      <c r="B1950" t="n">
+        <v>5</v>
+      </c>
+      <c r="C1950" t="n">
+        <v>20</v>
+      </c>
+      <c r="D1950" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E1950" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1950" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1950" t="n">
+        <v>30</v>
+      </c>
+      <c r="H1950" t="n">
+        <v>46</v>
+      </c>
+      <c r="I1950" t="n">
+        <v>57</v>
+      </c>
+      <c r="J1950" t="n">
+        <v>25</v>
+      </c>
+      <c r="K1950" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1951">
+      <c r="A1951" t="inlineStr">
+        <is>
+          <t>Powerball</t>
+        </is>
+      </c>
+      <c r="B1951" t="n">
+        <v>5</v>
+      </c>
+      <c r="C1951" t="n">
+        <v>23</v>
+      </c>
+      <c r="D1951" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E1951" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1951" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1951" t="n">
+        <v>41</v>
+      </c>
+      <c r="H1951" t="n">
+        <v>48</v>
+      </c>
+      <c r="I1951" t="n">
+        <v>66</v>
+      </c>
+      <c r="J1951" t="n">
+        <v>26</v>
+      </c>
+      <c r="K1951" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
perform mega million analysis
</commit_message>
<xml_diff>
--- a/powerball_game.xlsx
+++ b/powerball_game.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1949"/>
+  <dimension ref="A1:K1956"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -72141,6 +72141,265 @@
         <v>3</v>
       </c>
     </row>
+    <row r="1950">
+      <c r="A1950" t="inlineStr">
+        <is>
+          <t>Powerball</t>
+        </is>
+      </c>
+      <c r="B1950" t="n">
+        <v>6</v>
+      </c>
+      <c r="C1950" t="n">
+        <v>1</v>
+      </c>
+      <c r="D1950" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E1950" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1950" t="n">
+        <v>42</v>
+      </c>
+      <c r="G1950" t="n">
+        <v>47</v>
+      </c>
+      <c r="H1950" t="n">
+        <v>57</v>
+      </c>
+      <c r="I1950" t="n">
+        <v>58</v>
+      </c>
+      <c r="J1950" t="n">
+        <v>14</v>
+      </c>
+      <c r="K1950" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1951">
+      <c r="A1951" t="inlineStr">
+        <is>
+          <t>Powerball</t>
+        </is>
+      </c>
+      <c r="B1951" t="n">
+        <v>5</v>
+      </c>
+      <c r="C1951" t="n">
+        <v>30</v>
+      </c>
+      <c r="D1951" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E1951" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1951" t="n">
+        <v>27</v>
+      </c>
+      <c r="G1951" t="n">
+        <v>35</v>
+      </c>
+      <c r="H1951" t="n">
+        <v>44</v>
+      </c>
+      <c r="I1951" t="n">
+        <v>52</v>
+      </c>
+      <c r="J1951" t="n">
+        <v>12</v>
+      </c>
+      <c r="K1951" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1952">
+      <c r="A1952" t="inlineStr">
+        <is>
+          <t>Powerball</t>
+        </is>
+      </c>
+      <c r="B1952" t="n">
+        <v>5</v>
+      </c>
+      <c r="C1952" t="n">
+        <v>27</v>
+      </c>
+      <c r="D1952" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E1952" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1952" t="n">
+        <v>14</v>
+      </c>
+      <c r="G1952" t="n">
+        <v>21</v>
+      </c>
+      <c r="H1952" t="n">
+        <v>31</v>
+      </c>
+      <c r="I1952" t="n">
+        <v>51</v>
+      </c>
+      <c r="J1952" t="n">
+        <v>13</v>
+      </c>
+      <c r="K1952" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="1953">
+      <c r="A1953" t="inlineStr">
+        <is>
+          <t>Powerball</t>
+        </is>
+      </c>
+      <c r="B1953" t="n">
+        <v>5</v>
+      </c>
+      <c r="C1953" t="n">
+        <v>25</v>
+      </c>
+      <c r="D1953" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E1953" t="n">
+        <v>17</v>
+      </c>
+      <c r="F1953" t="n">
+        <v>32</v>
+      </c>
+      <c r="G1953" t="n">
+        <v>48</v>
+      </c>
+      <c r="H1953" t="n">
+        <v>60</v>
+      </c>
+      <c r="I1953" t="n">
+        <v>64</v>
+      </c>
+      <c r="J1953" t="n">
+        <v>10</v>
+      </c>
+      <c r="K1953" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1954">
+      <c r="A1954" t="inlineStr">
+        <is>
+          <t>Powerball</t>
+        </is>
+      </c>
+      <c r="B1954" t="n">
+        <v>5</v>
+      </c>
+      <c r="C1954" t="n">
+        <v>23</v>
+      </c>
+      <c r="D1954" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E1954" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1954" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1954" t="n">
+        <v>41</v>
+      </c>
+      <c r="H1954" t="n">
+        <v>48</v>
+      </c>
+      <c r="I1954" t="n">
+        <v>66</v>
+      </c>
+      <c r="J1954" t="n">
+        <v>26</v>
+      </c>
+      <c r="K1954" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="1955">
+      <c r="A1955" t="inlineStr">
+        <is>
+          <t>Powerball</t>
+        </is>
+      </c>
+      <c r="B1955" t="n">
+        <v>5</v>
+      </c>
+      <c r="C1955" t="n">
+        <v>20</v>
+      </c>
+      <c r="D1955" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E1955" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1955" t="n">
+        <v>28</v>
+      </c>
+      <c r="G1955" t="n">
+        <v>30</v>
+      </c>
+      <c r="H1955" t="n">
+        <v>46</v>
+      </c>
+      <c r="I1955" t="n">
+        <v>57</v>
+      </c>
+      <c r="J1955" t="n">
+        <v>25</v>
+      </c>
+      <c r="K1955" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="1956">
+      <c r="A1956" t="inlineStr">
+        <is>
+          <t>Powerball</t>
+        </is>
+      </c>
+      <c r="B1956" t="n">
+        <v>6</v>
+      </c>
+      <c r="C1956" t="n">
+        <v>3</v>
+      </c>
+      <c r="D1956" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E1956" t="n">
+        <v>14</v>
+      </c>
+      <c r="F1956" t="n">
+        <v>16</v>
+      </c>
+      <c r="G1956" t="n">
+        <v>38</v>
+      </c>
+      <c r="H1956" t="n">
+        <v>55</v>
+      </c>
+      <c r="I1956" t="n">
+        <v>64</v>
+      </c>
+      <c r="J1956" t="n">
+        <v>12</v>
+      </c>
+      <c r="K1956" t="n">
+        <v>3</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>